<commit_message>
Cotizacion Hardware y Software Actualizado
</commit_message>
<xml_diff>
--- a/Hardware/Cotizacion.xlsx
+++ b/Hardware/Cotizacion.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mlosada\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Debian\home\esneiderlg\repoVT\sga-unal-palmira\Hardware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5F4EE472-ED88-4A9F-9FB7-EB229025EF31}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62B92A5D-4845-467B-9A48-CFCADE346E7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7545" xr2:uid="{F7E60E79-78CA-45D4-AF1A-046033B5381E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{F7E60E79-78CA-45D4-AF1A-046033B5381E}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -21,12 +21,24 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="48">
   <si>
     <t>Modulo VT</t>
   </si>
@@ -127,10 +139,49 @@
     <t>WIKA 4-10 (0-100 psi)</t>
   </si>
   <si>
-    <t>ESPERA</t>
-  </si>
-  <si>
     <t>Sensor caudal a espera de limpieza</t>
+  </si>
+  <si>
+    <t>Sensor</t>
+  </si>
+  <si>
+    <t>Gateway</t>
+  </si>
+  <si>
+    <t>TOTAL X30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">total </t>
+  </si>
+  <si>
+    <t>Bateria</t>
+  </si>
+  <si>
+    <t>Suma Hardware</t>
+  </si>
+  <si>
+    <t>Suma Software</t>
+  </si>
+  <si>
+    <t>Envio  Hardware</t>
+  </si>
+  <si>
+    <t>Importacion</t>
+  </si>
+  <si>
+    <t>Mano de obra instalacion</t>
+  </si>
+  <si>
+    <t>Mano de obra Hardware</t>
+  </si>
+  <si>
+    <t>Sub Total</t>
+  </si>
+  <si>
+    <t>Total +  IVA</t>
+  </si>
+  <si>
+    <t>Utilidad VT</t>
   </si>
 </sst>
 </file>
@@ -179,11 +230,11 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Moneda" xfId="1" builtinId="4"/>
@@ -499,419 +550,566 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9516EE50-0B12-461A-96C2-5CA139EA51CB}">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.42578125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="H1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I1" s="1">
+        <f>B6+B18+B26</f>
+        <v>5482012</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="1">
         <f>Hoja2!C17</f>
-        <v>948110.54</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+        <v>962806</v>
+      </c>
+      <c r="H2" t="s">
+        <v>40</v>
+      </c>
+      <c r="I2" s="1">
+        <v>7500000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>25</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="1">
         <v>150000</v>
       </c>
       <c r="C3" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="H3" t="s">
+        <v>41</v>
+      </c>
+      <c r="I3" s="1">
+        <f>I1*0.12</f>
+        <v>657841.43999999994</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="1">
         <v>50000</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="H4" t="s">
+        <v>42</v>
+      </c>
+      <c r="I4" s="1">
+        <f>I1*0.35</f>
+        <v>1918704.2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>28</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="1">
         <v>200000</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="H5" t="s">
+        <v>44</v>
+      </c>
+      <c r="I5" s="1">
+        <v>650000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6" s="1">
         <f>SUM(B2:B5)</f>
-        <v>1348110.54</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+        <v>1362806</v>
+      </c>
+      <c r="H6" t="s">
+        <v>43</v>
+      </c>
+      <c r="I6" s="1">
+        <v>600000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>37</v>
+      </c>
+      <c r="H7" t="s">
+        <v>45</v>
+      </c>
+      <c r="I7" s="1">
+        <f>SUM(I1:I6)</f>
+        <v>16808557.640000001</v>
+      </c>
+      <c r="K7" s="2"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="H8" t="s">
+        <v>46</v>
+      </c>
+      <c r="I8" s="1">
+        <f>I7*1.2</f>
+        <v>20170269.168000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="H9" t="s">
+        <v>47</v>
+      </c>
+      <c r="I9" s="1">
+        <f>I8*1.2</f>
+        <v>24204323.001600001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>0</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B11" s="1">
         <f>Hoja2!C17</f>
-        <v>948110.54</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+        <v>962806</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>25</v>
       </c>
-      <c r="B12" s="2">
+      <c r="B12" s="1">
         <v>150000</v>
       </c>
       <c r="C12" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>32</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="1">
+        <f>Hoja2!R5</f>
+        <v>1330000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>27</v>
       </c>
-      <c r="B16" s="2">
+      <c r="B16" s="1">
         <v>100000</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>31</v>
       </c>
-      <c r="B17" s="2">
+      <c r="B17" s="1">
         <v>120000</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>29</v>
       </c>
-      <c r="B18" s="2">
+      <c r="B18" s="1">
         <f>SUM(B11:B17)</f>
-        <v>1318110.54</v>
+        <v>2662806</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>0</v>
+      </c>
+      <c r="B22" s="1">
+        <f>Hoja2!G17</f>
+        <v>1056400</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>38</v>
+      </c>
+      <c r="B23" s="1">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>27</v>
+      </c>
+      <c r="B24" s="1">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>28</v>
+      </c>
+      <c r="B25" s="1">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>29</v>
+      </c>
+      <c r="B26" s="1">
+        <f>SUM(B22:B25)</f>
+        <v>1456400</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A21:D21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F99908F6-0BAC-4562-AE05-2FE90F87F37D}">
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:R17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="E1" s="1" t="s">
+      <c r="B1" s="3"/>
+      <c r="E1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="F1" s="1"/>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="F1" s="3"/>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="1">
         <v>4.37</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="2">
         <f>B2*K$2</f>
-        <v>16352.54</v>
+        <v>16606</v>
       </c>
       <c r="E2" t="s">
         <v>17</v>
       </c>
-      <c r="F2" s="2">
+      <c r="F2" s="1">
         <v>120</v>
       </c>
-      <c r="G2" s="3">
+      <c r="G2" s="2">
         <f>F2*K$2</f>
-        <v>449040</v>
+        <v>456000</v>
       </c>
       <c r="J2" t="s">
         <v>10</v>
       </c>
       <c r="K2">
-        <v>3742</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+        <v>3800</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="1">
         <v>18</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="2">
         <f t="shared" ref="C3:C14" si="0">B3*K$2</f>
-        <v>67356</v>
+        <v>68400</v>
       </c>
       <c r="E3" t="s">
         <v>18</v>
       </c>
-      <c r="F3" s="2">
+      <c r="F3" s="1">
         <v>18</v>
       </c>
-      <c r="G3" s="3">
-        <f t="shared" ref="G3:G9" si="1">F3*K$2</f>
-        <v>67356</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="G3" s="2">
+        <f t="shared" ref="G3:G8" si="1">F3*K$2</f>
+        <v>68400</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="1">
         <v>7</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="2">
         <f t="shared" si="0"/>
-        <v>26194</v>
+        <v>26600</v>
       </c>
       <c r="E4" t="s">
         <v>19</v>
       </c>
-      <c r="F4" s="2">
+      <c r="F4" s="1">
         <v>20</v>
       </c>
-      <c r="G4" s="3">
+      <c r="G4" s="2">
         <f t="shared" si="1"/>
-        <v>74840</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+        <v>76000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="1">
         <v>5</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="2">
         <f t="shared" si="0"/>
-        <v>18710</v>
+        <v>19000</v>
       </c>
       <c r="E5" t="s">
         <v>20</v>
       </c>
-      <c r="F5" s="2">
+      <c r="F5" s="1">
         <v>25</v>
       </c>
-      <c r="G5" s="3">
+      <c r="G5" s="2">
         <f t="shared" si="1"/>
-        <v>93550</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+        <v>95000</v>
+      </c>
+      <c r="P5" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q5" s="1">
+        <v>350</v>
+      </c>
+      <c r="R5" s="2">
+        <f>K2*Q5</f>
+        <v>1330000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6" s="1">
         <v>30</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="2">
         <f t="shared" si="0"/>
-        <v>112260</v>
+        <v>114000</v>
       </c>
       <c r="E6" t="s">
         <v>21</v>
       </c>
-      <c r="F6" s="2">
+      <c r="F6" s="1">
         <v>12</v>
       </c>
-      <c r="G6" s="3">
+      <c r="G6" s="2">
         <f t="shared" si="1"/>
-        <v>44904</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+        <v>45600</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7" s="1">
         <v>5</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" s="2">
         <f t="shared" si="0"/>
-        <v>18710</v>
+        <v>19000</v>
       </c>
       <c r="E7" t="s">
         <v>22</v>
       </c>
-      <c r="F7" s="2">
+      <c r="F7" s="1">
         <v>23</v>
       </c>
-      <c r="G7" s="3">
+      <c r="G7" s="2">
         <f t="shared" si="1"/>
-        <v>86066</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+        <v>87400</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="2">
+      <c r="B8" s="1">
         <v>5</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C8" s="2">
         <f t="shared" si="0"/>
-        <v>18710</v>
+        <v>19000</v>
       </c>
       <c r="E8" t="s">
         <v>23</v>
       </c>
-      <c r="F8" s="2">
+      <c r="F8" s="1">
         <v>60</v>
       </c>
-      <c r="G8" s="3">
+      <c r="G8" s="2">
         <f t="shared" si="1"/>
-        <v>224520</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+        <v>228000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="2">
+      <c r="B9" s="1">
         <v>20</v>
       </c>
-      <c r="C9" s="3">
+      <c r="C9" s="2">
         <f t="shared" si="0"/>
-        <v>74840</v>
-      </c>
-      <c r="F9" s="2"/>
-      <c r="G9" s="3"/>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+        <v>76000</v>
+      </c>
+      <c r="F9" s="1"/>
+      <c r="G9" s="2"/>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="2">
+      <c r="B10" s="1">
         <v>60</v>
       </c>
-      <c r="C10" s="3">
+      <c r="C10" s="2">
         <f t="shared" si="0"/>
-        <v>224520</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+        <v>228000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B11" s="1">
         <f>5+18</f>
         <v>23</v>
       </c>
-      <c r="C11" s="3">
+      <c r="C11" s="2">
         <f t="shared" si="0"/>
-        <v>86066</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+        <v>87400</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="2">
+      <c r="B12" s="1">
         <v>6</v>
       </c>
-      <c r="C12" s="3">
+      <c r="C12" s="2">
         <f t="shared" si="0"/>
-        <v>22452</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+        <v>22800</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="2">
+      <c r="B13" s="1">
         <v>30</v>
       </c>
-      <c r="C13" s="3">
+      <c r="C13" s="2">
         <f t="shared" si="0"/>
-        <v>112260</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+        <v>114000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="2">
+      <c r="B14" s="1">
         <v>40</v>
       </c>
-      <c r="C14" s="3">
+      <c r="C14" s="2">
         <f t="shared" si="0"/>
-        <v>149680</v>
+        <v>152000</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>13</v>
       </c>
-      <c r="B17" s="2">
+      <c r="B17" s="1">
         <f>SUM(B2:B16)</f>
         <v>253.37</v>
       </c>
-      <c r="C17" s="3">
+      <c r="C17" s="2">
         <f>SUM(C2:C16)</f>
-        <v>948110.54</v>
+        <v>962806</v>
       </c>
       <c r="E17" t="s">
         <v>13</v>
       </c>
-      <c r="F17" s="2">
+      <c r="F17" s="1">
         <f>SUM(F2:F16)</f>
         <v>278</v>
       </c>
-      <c r="G17" s="3">
+      <c r="G17" s="2">
         <f>SUM(G2:G16)</f>
-        <v>1040276</v>
+        <v>1056400</v>
       </c>
     </row>
   </sheetData>

</xml_diff>